<commit_message>
Corrige le calendrier : mois 1 = FundedNext seul (payout net 700), achats à partir du mois 2
Les achats sont financés par l'argent accumulé des mois précédents, donc le
premier mois ne détient que le compte de départ ; le capital affiché au mois 1
est 10 000 et le payout net 700.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XpnEpdwNF8V8azepdqLgDD
</commit_message>
<xml_diff>
--- a/docs/plan-scaling-diversifie.xlsx
+++ b/docs/plan-scaling-diversifie.xlsx
@@ -254,7 +254,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Simulation'!H1</f>
+              <f>'Simulation'!F1</f>
             </strRef>
           </tx>
           <spPr>
@@ -277,7 +277,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Simulation'!$H$2:$H$61</f>
+              <f>'Simulation'!$F$2:$F$61</f>
             </numRef>
           </val>
         </ser>
@@ -286,7 +286,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Simulation'!I1</f>
+              <f>'Simulation'!G1</f>
             </strRef>
           </tx>
           <spPr>
@@ -309,7 +309,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Simulation'!$I$2:$I$61</f>
+              <f>'Simulation'!$G$2:$G$61</f>
             </numRef>
           </val>
         </ser>
@@ -390,7 +390,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Revenu mensuel potentiel</a:t>
+              <a:t>Revenu mensuel net</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -522,7 +522,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Simulation'!E1</f>
+              <f>'Simulation'!B1</f>
             </strRef>
           </tx>
           <spPr>
@@ -545,7 +545,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Simulation'!$E$2:$E$61</f>
+              <f>'Simulation'!$B$2:$B$61</f>
             </numRef>
           </val>
         </ser>
@@ -11647,20 +11647,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -11671,52 +11670,47 @@
       </c>
       <c r="B1" s="9" t="inlineStr">
         <is>
-          <t>Capital financé début ($)</t>
+          <t>Firmes détenues ce mois</t>
         </is>
       </c>
       <c r="C1" s="9" t="inlineStr">
         <is>
+          <t>Capital financé actif ($)</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Payout brut du mois ($)</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
           <t>Payout net du mois ($)</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
-        <is>
-          <t>Réinvesti cumulé ($)</t>
-        </is>
-      </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>Firmes détenues</t>
-        </is>
-      </c>
       <c r="F1" s="9" t="inlineStr">
         <is>
+          <t>dont CFD ($)</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>dont Futures ($)</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>Payout net cumulé ($)</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
           <t>Nouvelles firmes ce mois</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
-        <is>
-          <t>Capital financé fin ($)</t>
-        </is>
-      </c>
-      <c r="H1" s="9" t="inlineStr">
-        <is>
-          <t>dont CFD ($)</t>
-        </is>
-      </c>
-      <c r="I1" s="9" t="inlineStr">
-        <is>
-          <t>dont Futures ($)</t>
-        </is>
-      </c>
       <c r="J1" s="9" t="inlineStr">
         <is>
-          <t>Revenu mensuel potentiel ($)</t>
-        </is>
-      </c>
-      <c r="K1" s="9" t="inlineStr">
-        <is>
-          <t>Trésorerie ($)</t>
+          <t>Revenu mensuel net ($)</t>
         </is>
       </c>
     </row>
@@ -11724,44 +11718,40 @@
       <c r="A2" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="12">
-        <f>Paramètres!$B$5</f>
-        <v/>
-      </c>
-      <c r="C2" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,0),0))*Paramètres!$B$3</f>
+      <c r="B2" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;0))</f>
+        <v/>
+      </c>
+      <c r="C2" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B2),0)</f>
         <v/>
       </c>
       <c r="D2" s="12">
-        <f>C2</f>
-        <v/>
-      </c>
-      <c r="E2" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D2))</f>
-        <v/>
-      </c>
-      <c r="F2" s="10">
-        <f>E2-0</f>
-        <v/>
-      </c>
-      <c r="G2" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E2),0)</f>
+        <f>C2*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E2" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B2),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F2" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B2,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G2" s="12">
+        <f>C2-F2</f>
         <v/>
       </c>
       <c r="H2" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E2,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I2" s="12">
-        <f>G2-H2</f>
-        <v/>
-      </c>
-      <c r="J2" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E2),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K2" s="12">
-        <f>D2-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E2),0)</f>
+        <f>E2</f>
+        <v/>
+      </c>
+      <c r="I2" s="10">
+        <f>B2</f>
+        <v/>
+      </c>
+      <c r="J2" s="12">
+        <f>E2</f>
         <v/>
       </c>
     </row>
@@ -11769,44 +11759,40 @@
       <c r="A3" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="12">
-        <f>G2</f>
-        <v/>
-      </c>
-      <c r="C3" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E2),0))*Paramètres!$B$3</f>
+      <c r="B3" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H2))</f>
+        <v/>
+      </c>
+      <c r="C3" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B3),0)</f>
         <v/>
       </c>
       <c r="D3" s="12">
-        <f>D2+C3</f>
-        <v/>
-      </c>
-      <c r="E3" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D3))</f>
-        <v/>
-      </c>
-      <c r="F3" s="10">
-        <f>E3-E2</f>
-        <v/>
-      </c>
-      <c r="G3" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E3),0)</f>
+        <f>C3*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E3" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B3),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F3" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B3,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G3" s="12">
+        <f>C3-F3</f>
         <v/>
       </c>
       <c r="H3" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E3,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I3" s="12">
-        <f>G3-H3</f>
-        <v/>
-      </c>
-      <c r="J3" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E3),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K3" s="12">
-        <f>D3-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E3),0)</f>
+        <f>H2+E3</f>
+        <v/>
+      </c>
+      <c r="I3" s="10">
+        <f>B3-B2</f>
+        <v/>
+      </c>
+      <c r="J3" s="12">
+        <f>E3</f>
         <v/>
       </c>
     </row>
@@ -11814,44 +11800,40 @@
       <c r="A4" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="12">
-        <f>G3</f>
-        <v/>
-      </c>
-      <c r="C4" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E3),0))*Paramètres!$B$3</f>
+      <c r="B4" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H3))</f>
+        <v/>
+      </c>
+      <c r="C4" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B4),0)</f>
         <v/>
       </c>
       <c r="D4" s="12">
-        <f>D3+C4</f>
-        <v/>
-      </c>
-      <c r="E4" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D4))</f>
-        <v/>
-      </c>
-      <c r="F4" s="10">
-        <f>E4-E3</f>
-        <v/>
-      </c>
-      <c r="G4" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E4),0)</f>
+        <f>C4*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E4" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B4),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F4" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B4,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G4" s="12">
+        <f>C4-F4</f>
         <v/>
       </c>
       <c r="H4" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E4,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I4" s="12">
-        <f>G4-H4</f>
-        <v/>
-      </c>
-      <c r="J4" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E4),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K4" s="12">
-        <f>D4-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E4),0)</f>
+        <f>H3+E4</f>
+        <v/>
+      </c>
+      <c r="I4" s="10">
+        <f>B4-B3</f>
+        <v/>
+      </c>
+      <c r="J4" s="12">
+        <f>E4</f>
         <v/>
       </c>
     </row>
@@ -11859,44 +11841,40 @@
       <c r="A5" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="12">
-        <f>G4</f>
-        <v/>
-      </c>
-      <c r="C5" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E4),0))*Paramètres!$B$3</f>
+      <c r="B5" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H4))</f>
+        <v/>
+      </c>
+      <c r="C5" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B5),0)</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>D4+C5</f>
-        <v/>
-      </c>
-      <c r="E5" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D5))</f>
-        <v/>
-      </c>
-      <c r="F5" s="10">
-        <f>E5-E4</f>
-        <v/>
-      </c>
-      <c r="G5" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E5),0)</f>
+        <f>C5*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E5" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B5),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F5" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B5,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G5" s="12">
+        <f>C5-F5</f>
         <v/>
       </c>
       <c r="H5" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E5,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I5" s="12">
-        <f>G5-H5</f>
-        <v/>
-      </c>
-      <c r="J5" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E5),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K5" s="12">
-        <f>D5-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E5),0)</f>
+        <f>H4+E5</f>
+        <v/>
+      </c>
+      <c r="I5" s="10">
+        <f>B5-B4</f>
+        <v/>
+      </c>
+      <c r="J5" s="12">
+        <f>E5</f>
         <v/>
       </c>
     </row>
@@ -11904,44 +11882,40 @@
       <c r="A6" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="12">
-        <f>G5</f>
-        <v/>
-      </c>
-      <c r="C6" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E5),0))*Paramètres!$B$3</f>
+      <c r="B6" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H5))</f>
+        <v/>
+      </c>
+      <c r="C6" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B6),0)</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>D5+C6</f>
-        <v/>
-      </c>
-      <c r="E6" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D6))</f>
-        <v/>
-      </c>
-      <c r="F6" s="10">
-        <f>E6-E5</f>
-        <v/>
-      </c>
-      <c r="G6" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E6),0)</f>
+        <f>C6*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E6" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B6),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F6" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B6,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G6" s="12">
+        <f>C6-F6</f>
         <v/>
       </c>
       <c r="H6" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E6,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I6" s="12">
-        <f>G6-H6</f>
-        <v/>
-      </c>
-      <c r="J6" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E6),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K6" s="12">
-        <f>D6-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E6),0)</f>
+        <f>H5+E6</f>
+        <v/>
+      </c>
+      <c r="I6" s="10">
+        <f>B6-B5</f>
+        <v/>
+      </c>
+      <c r="J6" s="12">
+        <f>E6</f>
         <v/>
       </c>
     </row>
@@ -11949,44 +11923,40 @@
       <c r="A7" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="12">
-        <f>G6</f>
-        <v/>
-      </c>
-      <c r="C7" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E6),0))*Paramètres!$B$3</f>
+      <c r="B7" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H6))</f>
+        <v/>
+      </c>
+      <c r="C7" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B7),0)</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>D6+C7</f>
-        <v/>
-      </c>
-      <c r="E7" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D7))</f>
-        <v/>
-      </c>
-      <c r="F7" s="10">
-        <f>E7-E6</f>
-        <v/>
-      </c>
-      <c r="G7" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E7),0)</f>
+        <f>C7*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E7" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B7),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F7" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B7,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G7" s="12">
+        <f>C7-F7</f>
         <v/>
       </c>
       <c r="H7" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E7,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I7" s="12">
-        <f>G7-H7</f>
-        <v/>
-      </c>
-      <c r="J7" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E7),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K7" s="12">
-        <f>D7-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E7),0)</f>
+        <f>H6+E7</f>
+        <v/>
+      </c>
+      <c r="I7" s="10">
+        <f>B7-B6</f>
+        <v/>
+      </c>
+      <c r="J7" s="12">
+        <f>E7</f>
         <v/>
       </c>
     </row>
@@ -11994,44 +11964,40 @@
       <c r="A8" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="12">
-        <f>G7</f>
-        <v/>
-      </c>
-      <c r="C8" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E7),0))*Paramètres!$B$3</f>
+      <c r="B8" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H7))</f>
+        <v/>
+      </c>
+      <c r="C8" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B8),0)</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>D7+C8</f>
-        <v/>
-      </c>
-      <c r="E8" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D8))</f>
-        <v/>
-      </c>
-      <c r="F8" s="10">
-        <f>E8-E7</f>
-        <v/>
-      </c>
-      <c r="G8" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E8),0)</f>
+        <f>C8*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E8" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B8),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F8" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B8,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G8" s="12">
+        <f>C8-F8</f>
         <v/>
       </c>
       <c r="H8" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E8,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I8" s="12">
-        <f>G8-H8</f>
-        <v/>
-      </c>
-      <c r="J8" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E8),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K8" s="12">
-        <f>D8-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E8),0)</f>
+        <f>H7+E8</f>
+        <v/>
+      </c>
+      <c r="I8" s="10">
+        <f>B8-B7</f>
+        <v/>
+      </c>
+      <c r="J8" s="12">
+        <f>E8</f>
         <v/>
       </c>
     </row>
@@ -12039,44 +12005,40 @@
       <c r="A9" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="12">
-        <f>G8</f>
-        <v/>
-      </c>
-      <c r="C9" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E8),0))*Paramètres!$B$3</f>
+      <c r="B9" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H8))</f>
+        <v/>
+      </c>
+      <c r="C9" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B9),0)</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>D8+C9</f>
-        <v/>
-      </c>
-      <c r="E9" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D9))</f>
-        <v/>
-      </c>
-      <c r="F9" s="10">
-        <f>E9-E8</f>
-        <v/>
-      </c>
-      <c r="G9" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E9),0)</f>
+        <f>C9*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E9" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B9),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F9" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B9,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G9" s="12">
+        <f>C9-F9</f>
         <v/>
       </c>
       <c r="H9" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E9,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I9" s="12">
-        <f>G9-H9</f>
-        <v/>
-      </c>
-      <c r="J9" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E9),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K9" s="12">
-        <f>D9-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E9),0)</f>
+        <f>H8+E9</f>
+        <v/>
+      </c>
+      <c r="I9" s="10">
+        <f>B9-B8</f>
+        <v/>
+      </c>
+      <c r="J9" s="12">
+        <f>E9</f>
         <v/>
       </c>
     </row>
@@ -12084,44 +12046,40 @@
       <c r="A10" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="12">
-        <f>G9</f>
-        <v/>
-      </c>
-      <c r="C10" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E9),0))*Paramètres!$B$3</f>
+      <c r="B10" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H9))</f>
+        <v/>
+      </c>
+      <c r="C10" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B10),0)</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>D9+C10</f>
-        <v/>
-      </c>
-      <c r="E10" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D10))</f>
-        <v/>
-      </c>
-      <c r="F10" s="10">
-        <f>E10-E9</f>
-        <v/>
-      </c>
-      <c r="G10" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E10),0)</f>
+        <f>C10*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E10" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B10),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F10" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B10,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G10" s="12">
+        <f>C10-F10</f>
         <v/>
       </c>
       <c r="H10" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E10,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I10" s="12">
-        <f>G10-H10</f>
-        <v/>
-      </c>
-      <c r="J10" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E10),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K10" s="12">
-        <f>D10-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E10),0)</f>
+        <f>H9+E10</f>
+        <v/>
+      </c>
+      <c r="I10" s="10">
+        <f>B10-B9</f>
+        <v/>
+      </c>
+      <c r="J10" s="12">
+        <f>E10</f>
         <v/>
       </c>
     </row>
@@ -12129,44 +12087,40 @@
       <c r="A11" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="12">
-        <f>G10</f>
-        <v/>
-      </c>
-      <c r="C11" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E10),0))*Paramètres!$B$3</f>
+      <c r="B11" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H10))</f>
+        <v/>
+      </c>
+      <c r="C11" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B11),0)</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>D10+C11</f>
-        <v/>
-      </c>
-      <c r="E11" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D11))</f>
-        <v/>
-      </c>
-      <c r="F11" s="10">
-        <f>E11-E10</f>
-        <v/>
-      </c>
-      <c r="G11" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E11),0)</f>
+        <f>C11*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E11" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B11),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F11" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B11,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G11" s="12">
+        <f>C11-F11</f>
         <v/>
       </c>
       <c r="H11" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E11,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I11" s="12">
-        <f>G11-H11</f>
-        <v/>
-      </c>
-      <c r="J11" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E11),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K11" s="12">
-        <f>D11-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E11),0)</f>
+        <f>H10+E11</f>
+        <v/>
+      </c>
+      <c r="I11" s="10">
+        <f>B11-B10</f>
+        <v/>
+      </c>
+      <c r="J11" s="12">
+        <f>E11</f>
         <v/>
       </c>
     </row>
@@ -12174,44 +12128,40 @@
       <c r="A12" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="12">
-        <f>G11</f>
-        <v/>
-      </c>
-      <c r="C12" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E11),0))*Paramètres!$B$3</f>
+      <c r="B12" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H11))</f>
+        <v/>
+      </c>
+      <c r="C12" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B12),0)</f>
         <v/>
       </c>
       <c r="D12" s="12">
-        <f>D11+C12</f>
-        <v/>
-      </c>
-      <c r="E12" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D12))</f>
-        <v/>
-      </c>
-      <c r="F12" s="10">
-        <f>E12-E11</f>
-        <v/>
-      </c>
-      <c r="G12" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E12),0)</f>
+        <f>C12*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E12" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B12),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F12" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B12,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G12" s="12">
+        <f>C12-F12</f>
         <v/>
       </c>
       <c r="H12" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E12,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I12" s="12">
-        <f>G12-H12</f>
-        <v/>
-      </c>
-      <c r="J12" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E12),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K12" s="12">
-        <f>D12-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E12),0)</f>
+        <f>H11+E12</f>
+        <v/>
+      </c>
+      <c r="I12" s="10">
+        <f>B12-B11</f>
+        <v/>
+      </c>
+      <c r="J12" s="12">
+        <f>E12</f>
         <v/>
       </c>
     </row>
@@ -12219,44 +12169,40 @@
       <c r="A13" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="12">
-        <f>G12</f>
-        <v/>
-      </c>
-      <c r="C13" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E12),0))*Paramètres!$B$3</f>
+      <c r="B13" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H12))</f>
+        <v/>
+      </c>
+      <c r="C13" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B13),0)</f>
         <v/>
       </c>
       <c r="D13" s="12">
-        <f>D12+C13</f>
-        <v/>
-      </c>
-      <c r="E13" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D13))</f>
-        <v/>
-      </c>
-      <c r="F13" s="10">
-        <f>E13-E12</f>
-        <v/>
-      </c>
-      <c r="G13" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E13),0)</f>
+        <f>C13*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E13" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B13),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F13" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B13,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G13" s="12">
+        <f>C13-F13</f>
         <v/>
       </c>
       <c r="H13" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E13,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I13" s="12">
-        <f>G13-H13</f>
-        <v/>
-      </c>
-      <c r="J13" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E13),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K13" s="12">
-        <f>D13-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E13),0)</f>
+        <f>H12+E13</f>
+        <v/>
+      </c>
+      <c r="I13" s="10">
+        <f>B13-B12</f>
+        <v/>
+      </c>
+      <c r="J13" s="12">
+        <f>E13</f>
         <v/>
       </c>
     </row>
@@ -12264,44 +12210,40 @@
       <c r="A14" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="12">
-        <f>G13</f>
-        <v/>
-      </c>
-      <c r="C14" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E13),0))*Paramètres!$B$3</f>
+      <c r="B14" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H13))</f>
+        <v/>
+      </c>
+      <c r="C14" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B14),0)</f>
         <v/>
       </c>
       <c r="D14" s="12">
-        <f>D13+C14</f>
-        <v/>
-      </c>
-      <c r="E14" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D14))</f>
-        <v/>
-      </c>
-      <c r="F14" s="10">
-        <f>E14-E13</f>
-        <v/>
-      </c>
-      <c r="G14" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E14),0)</f>
+        <f>C14*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E14" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B14),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F14" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B14,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G14" s="12">
+        <f>C14-F14</f>
         <v/>
       </c>
       <c r="H14" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E14,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I14" s="12">
-        <f>G14-H14</f>
-        <v/>
-      </c>
-      <c r="J14" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E14),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K14" s="12">
-        <f>D14-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E14),0)</f>
+        <f>H13+E14</f>
+        <v/>
+      </c>
+      <c r="I14" s="10">
+        <f>B14-B13</f>
+        <v/>
+      </c>
+      <c r="J14" s="12">
+        <f>E14</f>
         <v/>
       </c>
     </row>
@@ -12309,44 +12251,40 @@
       <c r="A15" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="12">
-        <f>G14</f>
-        <v/>
-      </c>
-      <c r="C15" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E14),0))*Paramètres!$B$3</f>
+      <c r="B15" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H14))</f>
+        <v/>
+      </c>
+      <c r="C15" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B15),0)</f>
         <v/>
       </c>
       <c r="D15" s="12">
-        <f>D14+C15</f>
-        <v/>
-      </c>
-      <c r="E15" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D15))</f>
-        <v/>
-      </c>
-      <c r="F15" s="10">
-        <f>E15-E14</f>
-        <v/>
-      </c>
-      <c r="G15" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E15),0)</f>
+        <f>C15*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E15" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B15),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F15" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B15,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G15" s="12">
+        <f>C15-F15</f>
         <v/>
       </c>
       <c r="H15" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E15,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I15" s="12">
-        <f>G15-H15</f>
-        <v/>
-      </c>
-      <c r="J15" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E15),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K15" s="12">
-        <f>D15-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E15),0)</f>
+        <f>H14+E15</f>
+        <v/>
+      </c>
+      <c r="I15" s="10">
+        <f>B15-B14</f>
+        <v/>
+      </c>
+      <c r="J15" s="12">
+        <f>E15</f>
         <v/>
       </c>
     </row>
@@ -12354,44 +12292,40 @@
       <c r="A16" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="12">
-        <f>G15</f>
-        <v/>
-      </c>
-      <c r="C16" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E15),0))*Paramètres!$B$3</f>
+      <c r="B16" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H15))</f>
+        <v/>
+      </c>
+      <c r="C16" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B16),0)</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>D15+C16</f>
-        <v/>
-      </c>
-      <c r="E16" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D16))</f>
-        <v/>
-      </c>
-      <c r="F16" s="10">
-        <f>E16-E15</f>
-        <v/>
-      </c>
-      <c r="G16" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E16),0)</f>
+        <f>C16*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E16" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B16),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F16" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B16,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G16" s="12">
+        <f>C16-F16</f>
         <v/>
       </c>
       <c r="H16" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E16,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I16" s="12">
-        <f>G16-H16</f>
-        <v/>
-      </c>
-      <c r="J16" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E16),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K16" s="12">
-        <f>D16-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E16),0)</f>
+        <f>H15+E16</f>
+        <v/>
+      </c>
+      <c r="I16" s="10">
+        <f>B16-B15</f>
+        <v/>
+      </c>
+      <c r="J16" s="12">
+        <f>E16</f>
         <v/>
       </c>
     </row>
@@ -12399,44 +12333,40 @@
       <c r="A17" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="12">
-        <f>G16</f>
-        <v/>
-      </c>
-      <c r="C17" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E16),0))*Paramètres!$B$3</f>
+      <c r="B17" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H16))</f>
+        <v/>
+      </c>
+      <c r="C17" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B17),0)</f>
         <v/>
       </c>
       <c r="D17" s="12">
-        <f>D16+C17</f>
-        <v/>
-      </c>
-      <c r="E17" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D17))</f>
-        <v/>
-      </c>
-      <c r="F17" s="10">
-        <f>E17-E16</f>
-        <v/>
-      </c>
-      <c r="G17" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E17),0)</f>
+        <f>C17*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E17" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B17),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F17" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B17,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G17" s="12">
+        <f>C17-F17</f>
         <v/>
       </c>
       <c r="H17" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E17,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I17" s="12">
-        <f>G17-H17</f>
-        <v/>
-      </c>
-      <c r="J17" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E17),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K17" s="12">
-        <f>D17-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E17),0)</f>
+        <f>H16+E17</f>
+        <v/>
+      </c>
+      <c r="I17" s="10">
+        <f>B17-B16</f>
+        <v/>
+      </c>
+      <c r="J17" s="12">
+        <f>E17</f>
         <v/>
       </c>
     </row>
@@ -12444,44 +12374,40 @@
       <c r="A18" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="12">
-        <f>G17</f>
-        <v/>
-      </c>
-      <c r="C18" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E17),0))*Paramètres!$B$3</f>
+      <c r="B18" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H17))</f>
+        <v/>
+      </c>
+      <c r="C18" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B18),0)</f>
         <v/>
       </c>
       <c r="D18" s="12">
-        <f>D17+C18</f>
-        <v/>
-      </c>
-      <c r="E18" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D18))</f>
-        <v/>
-      </c>
-      <c r="F18" s="10">
-        <f>E18-E17</f>
-        <v/>
-      </c>
-      <c r="G18" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E18),0)</f>
+        <f>C18*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E18" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B18),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F18" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B18,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G18" s="12">
+        <f>C18-F18</f>
         <v/>
       </c>
       <c r="H18" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E18,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I18" s="12">
-        <f>G18-H18</f>
-        <v/>
-      </c>
-      <c r="J18" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E18),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K18" s="12">
-        <f>D18-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E18),0)</f>
+        <f>H17+E18</f>
+        <v/>
+      </c>
+      <c r="I18" s="10">
+        <f>B18-B17</f>
+        <v/>
+      </c>
+      <c r="J18" s="12">
+        <f>E18</f>
         <v/>
       </c>
     </row>
@@ -12489,44 +12415,40 @@
       <c r="A19" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="12">
-        <f>G18</f>
-        <v/>
-      </c>
-      <c r="C19" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E18),0))*Paramètres!$B$3</f>
+      <c r="B19" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H18))</f>
+        <v/>
+      </c>
+      <c r="C19" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B19),0)</f>
         <v/>
       </c>
       <c r="D19" s="12">
-        <f>D18+C19</f>
-        <v/>
-      </c>
-      <c r="E19" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D19))</f>
-        <v/>
-      </c>
-      <c r="F19" s="10">
-        <f>E19-E18</f>
-        <v/>
-      </c>
-      <c r="G19" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E19),0)</f>
+        <f>C19*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E19" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B19),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F19" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B19,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G19" s="12">
+        <f>C19-F19</f>
         <v/>
       </c>
       <c r="H19" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E19,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I19" s="12">
-        <f>G19-H19</f>
-        <v/>
-      </c>
-      <c r="J19" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E19),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K19" s="12">
-        <f>D19-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E19),0)</f>
+        <f>H18+E19</f>
+        <v/>
+      </c>
+      <c r="I19" s="10">
+        <f>B19-B18</f>
+        <v/>
+      </c>
+      <c r="J19" s="12">
+        <f>E19</f>
         <v/>
       </c>
     </row>
@@ -12534,44 +12456,40 @@
       <c r="A20" s="10" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="12">
-        <f>G19</f>
-        <v/>
-      </c>
-      <c r="C20" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E19),0))*Paramètres!$B$3</f>
+      <c r="B20" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H19))</f>
+        <v/>
+      </c>
+      <c r="C20" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B20),0)</f>
         <v/>
       </c>
       <c r="D20" s="12">
-        <f>D19+C20</f>
-        <v/>
-      </c>
-      <c r="E20" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D20))</f>
-        <v/>
-      </c>
-      <c r="F20" s="10">
-        <f>E20-E19</f>
-        <v/>
-      </c>
-      <c r="G20" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E20),0)</f>
+        <f>C20*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E20" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B20),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F20" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B20,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G20" s="12">
+        <f>C20-F20</f>
         <v/>
       </c>
       <c r="H20" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E20,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I20" s="12">
-        <f>G20-H20</f>
-        <v/>
-      </c>
-      <c r="J20" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E20),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K20" s="12">
-        <f>D20-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E20),0)</f>
+        <f>H19+E20</f>
+        <v/>
+      </c>
+      <c r="I20" s="10">
+        <f>B20-B19</f>
+        <v/>
+      </c>
+      <c r="J20" s="12">
+        <f>E20</f>
         <v/>
       </c>
     </row>
@@ -12579,44 +12497,40 @@
       <c r="A21" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="12">
-        <f>G20</f>
-        <v/>
-      </c>
-      <c r="C21" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E20),0))*Paramètres!$B$3</f>
+      <c r="B21" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H20))</f>
+        <v/>
+      </c>
+      <c r="C21" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B21),0)</f>
         <v/>
       </c>
       <c r="D21" s="12">
-        <f>D20+C21</f>
-        <v/>
-      </c>
-      <c r="E21" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D21))</f>
-        <v/>
-      </c>
-      <c r="F21" s="10">
-        <f>E21-E20</f>
-        <v/>
-      </c>
-      <c r="G21" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E21),0)</f>
+        <f>C21*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E21" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B21),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F21" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B21,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G21" s="12">
+        <f>C21-F21</f>
         <v/>
       </c>
       <c r="H21" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E21,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I21" s="12">
-        <f>G21-H21</f>
-        <v/>
-      </c>
-      <c r="J21" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E21),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K21" s="12">
-        <f>D21-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E21),0)</f>
+        <f>H20+E21</f>
+        <v/>
+      </c>
+      <c r="I21" s="10">
+        <f>B21-B20</f>
+        <v/>
+      </c>
+      <c r="J21" s="12">
+        <f>E21</f>
         <v/>
       </c>
     </row>
@@ -12624,44 +12538,40 @@
       <c r="A22" s="10" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="12">
-        <f>G21</f>
-        <v/>
-      </c>
-      <c r="C22" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E21),0))*Paramètres!$B$3</f>
+      <c r="B22" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H21))</f>
+        <v/>
+      </c>
+      <c r="C22" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B22),0)</f>
         <v/>
       </c>
       <c r="D22" s="12">
-        <f>D21+C22</f>
-        <v/>
-      </c>
-      <c r="E22" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D22))</f>
-        <v/>
-      </c>
-      <c r="F22" s="10">
-        <f>E22-E21</f>
-        <v/>
-      </c>
-      <c r="G22" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E22),0)</f>
+        <f>C22*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E22" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B22),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F22" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B22,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G22" s="12">
+        <f>C22-F22</f>
         <v/>
       </c>
       <c r="H22" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E22,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I22" s="12">
-        <f>G22-H22</f>
-        <v/>
-      </c>
-      <c r="J22" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E22),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K22" s="12">
-        <f>D22-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E22),0)</f>
+        <f>H21+E22</f>
+        <v/>
+      </c>
+      <c r="I22" s="10">
+        <f>B22-B21</f>
+        <v/>
+      </c>
+      <c r="J22" s="12">
+        <f>E22</f>
         <v/>
       </c>
     </row>
@@ -12669,44 +12579,40 @@
       <c r="A23" s="10" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="12">
-        <f>G22</f>
-        <v/>
-      </c>
-      <c r="C23" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E22),0))*Paramètres!$B$3</f>
+      <c r="B23" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H22))</f>
+        <v/>
+      </c>
+      <c r="C23" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B23),0)</f>
         <v/>
       </c>
       <c r="D23" s="12">
-        <f>D22+C23</f>
-        <v/>
-      </c>
-      <c r="E23" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D23))</f>
-        <v/>
-      </c>
-      <c r="F23" s="10">
-        <f>E23-E22</f>
-        <v/>
-      </c>
-      <c r="G23" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E23),0)</f>
+        <f>C23*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E23" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B23),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F23" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B23,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G23" s="12">
+        <f>C23-F23</f>
         <v/>
       </c>
       <c r="H23" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E23,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I23" s="12">
-        <f>G23-H23</f>
-        <v/>
-      </c>
-      <c r="J23" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E23),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K23" s="12">
-        <f>D23-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E23),0)</f>
+        <f>H22+E23</f>
+        <v/>
+      </c>
+      <c r="I23" s="10">
+        <f>B23-B22</f>
+        <v/>
+      </c>
+      <c r="J23" s="12">
+        <f>E23</f>
         <v/>
       </c>
     </row>
@@ -12714,44 +12620,40 @@
       <c r="A24" s="10" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="12">
-        <f>G23</f>
-        <v/>
-      </c>
-      <c r="C24" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E23),0))*Paramètres!$B$3</f>
+      <c r="B24" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H23))</f>
+        <v/>
+      </c>
+      <c r="C24" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B24),0)</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>D23+C24</f>
-        <v/>
-      </c>
-      <c r="E24" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D24))</f>
-        <v/>
-      </c>
-      <c r="F24" s="10">
-        <f>E24-E23</f>
-        <v/>
-      </c>
-      <c r="G24" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E24),0)</f>
+        <f>C24*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E24" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B24),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F24" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B24,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G24" s="12">
+        <f>C24-F24</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E24,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I24" s="12">
-        <f>G24-H24</f>
-        <v/>
-      </c>
-      <c r="J24" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E24),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K24" s="12">
-        <f>D24-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E24),0)</f>
+        <f>H23+E24</f>
+        <v/>
+      </c>
+      <c r="I24" s="10">
+        <f>B24-B23</f>
+        <v/>
+      </c>
+      <c r="J24" s="12">
+        <f>E24</f>
         <v/>
       </c>
     </row>
@@ -12759,44 +12661,40 @@
       <c r="A25" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="12">
-        <f>G24</f>
-        <v/>
-      </c>
-      <c r="C25" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E24),0))*Paramètres!$B$3</f>
+      <c r="B25" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H24))</f>
+        <v/>
+      </c>
+      <c r="C25" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B25),0)</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>D24+C25</f>
-        <v/>
-      </c>
-      <c r="E25" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D25))</f>
-        <v/>
-      </c>
-      <c r="F25" s="10">
-        <f>E25-E24</f>
-        <v/>
-      </c>
-      <c r="G25" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E25),0)</f>
+        <f>C25*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E25" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B25),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F25" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B25,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G25" s="12">
+        <f>C25-F25</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E25,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I25" s="12">
-        <f>G25-H25</f>
-        <v/>
-      </c>
-      <c r="J25" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E25),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K25" s="12">
-        <f>D25-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E25),0)</f>
+        <f>H24+E25</f>
+        <v/>
+      </c>
+      <c r="I25" s="10">
+        <f>B25-B24</f>
+        <v/>
+      </c>
+      <c r="J25" s="12">
+        <f>E25</f>
         <v/>
       </c>
     </row>
@@ -12804,44 +12702,40 @@
       <c r="A26" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="12">
-        <f>G25</f>
-        <v/>
-      </c>
-      <c r="C26" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E25),0))*Paramètres!$B$3</f>
+      <c r="B26" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H25))</f>
+        <v/>
+      </c>
+      <c r="C26" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B26),0)</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>D25+C26</f>
-        <v/>
-      </c>
-      <c r="E26" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D26))</f>
-        <v/>
-      </c>
-      <c r="F26" s="10">
-        <f>E26-E25</f>
-        <v/>
-      </c>
-      <c r="G26" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E26),0)</f>
+        <f>C26*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E26" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B26),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F26" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B26,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G26" s="12">
+        <f>C26-F26</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E26,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I26" s="12">
-        <f>G26-H26</f>
-        <v/>
-      </c>
-      <c r="J26" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E26),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K26" s="12">
-        <f>D26-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E26),0)</f>
+        <f>H25+E26</f>
+        <v/>
+      </c>
+      <c r="I26" s="10">
+        <f>B26-B25</f>
+        <v/>
+      </c>
+      <c r="J26" s="12">
+        <f>E26</f>
         <v/>
       </c>
     </row>
@@ -12849,44 +12743,40 @@
       <c r="A27" s="10" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="12">
-        <f>G26</f>
-        <v/>
-      </c>
-      <c r="C27" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E26),0))*Paramètres!$B$3</f>
+      <c r="B27" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H26))</f>
+        <v/>
+      </c>
+      <c r="C27" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B27),0)</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>D26+C27</f>
-        <v/>
-      </c>
-      <c r="E27" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D27))</f>
-        <v/>
-      </c>
-      <c r="F27" s="10">
-        <f>E27-E26</f>
-        <v/>
-      </c>
-      <c r="G27" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E27),0)</f>
+        <f>C27*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E27" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B27),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F27" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B27,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G27" s="12">
+        <f>C27-F27</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E27,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I27" s="12">
-        <f>G27-H27</f>
-        <v/>
-      </c>
-      <c r="J27" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E27),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K27" s="12">
-        <f>D27-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E27),0)</f>
+        <f>H26+E27</f>
+        <v/>
+      </c>
+      <c r="I27" s="10">
+        <f>B27-B26</f>
+        <v/>
+      </c>
+      <c r="J27" s="12">
+        <f>E27</f>
         <v/>
       </c>
     </row>
@@ -12894,44 +12784,40 @@
       <c r="A28" s="10" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="12">
-        <f>G27</f>
-        <v/>
-      </c>
-      <c r="C28" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E27),0))*Paramètres!$B$3</f>
+      <c r="B28" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H27))</f>
+        <v/>
+      </c>
+      <c r="C28" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B28),0)</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>D27+C28</f>
-        <v/>
-      </c>
-      <c r="E28" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D28))</f>
-        <v/>
-      </c>
-      <c r="F28" s="10">
-        <f>E28-E27</f>
-        <v/>
-      </c>
-      <c r="G28" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E28),0)</f>
+        <f>C28*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E28" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B28),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F28" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B28,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G28" s="12">
+        <f>C28-F28</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E28,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I28" s="12">
-        <f>G28-H28</f>
-        <v/>
-      </c>
-      <c r="J28" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E28),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K28" s="12">
-        <f>D28-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E28),0)</f>
+        <f>H27+E28</f>
+        <v/>
+      </c>
+      <c r="I28" s="10">
+        <f>B28-B27</f>
+        <v/>
+      </c>
+      <c r="J28" s="12">
+        <f>E28</f>
         <v/>
       </c>
     </row>
@@ -12939,44 +12825,40 @@
       <c r="A29" s="10" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="12">
-        <f>G28</f>
-        <v/>
-      </c>
-      <c r="C29" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E28),0))*Paramètres!$B$3</f>
+      <c r="B29" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H28))</f>
+        <v/>
+      </c>
+      <c r="C29" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B29),0)</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>D28+C29</f>
-        <v/>
-      </c>
-      <c r="E29" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D29))</f>
-        <v/>
-      </c>
-      <c r="F29" s="10">
-        <f>E29-E28</f>
-        <v/>
-      </c>
-      <c r="G29" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E29),0)</f>
+        <f>C29*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E29" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B29),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F29" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B29,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G29" s="12">
+        <f>C29-F29</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E29,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I29" s="12">
-        <f>G29-H29</f>
-        <v/>
-      </c>
-      <c r="J29" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E29),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K29" s="12">
-        <f>D29-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E29),0)</f>
+        <f>H28+E29</f>
+        <v/>
+      </c>
+      <c r="I29" s="10">
+        <f>B29-B28</f>
+        <v/>
+      </c>
+      <c r="J29" s="12">
+        <f>E29</f>
         <v/>
       </c>
     </row>
@@ -12984,44 +12866,40 @@
       <c r="A30" s="10" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="12">
-        <f>G29</f>
-        <v/>
-      </c>
-      <c r="C30" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E29),0))*Paramètres!$B$3</f>
+      <c r="B30" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H29))</f>
+        <v/>
+      </c>
+      <c r="C30" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B30),0)</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>D29+C30</f>
-        <v/>
-      </c>
-      <c r="E30" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D30))</f>
-        <v/>
-      </c>
-      <c r="F30" s="10">
-        <f>E30-E29</f>
-        <v/>
-      </c>
-      <c r="G30" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E30),0)</f>
+        <f>C30*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E30" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B30),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F30" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B30,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G30" s="12">
+        <f>C30-F30</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E30,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I30" s="12">
-        <f>G30-H30</f>
-        <v/>
-      </c>
-      <c r="J30" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E30),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K30" s="12">
-        <f>D30-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E30),0)</f>
+        <f>H29+E30</f>
+        <v/>
+      </c>
+      <c r="I30" s="10">
+        <f>B30-B29</f>
+        <v/>
+      </c>
+      <c r="J30" s="12">
+        <f>E30</f>
         <v/>
       </c>
     </row>
@@ -13029,44 +12907,40 @@
       <c r="A31" s="10" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="12">
-        <f>G30</f>
-        <v/>
-      </c>
-      <c r="C31" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E30),0))*Paramètres!$B$3</f>
+      <c r="B31" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H30))</f>
+        <v/>
+      </c>
+      <c r="C31" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B31),0)</f>
         <v/>
       </c>
       <c r="D31" s="12">
-        <f>D30+C31</f>
-        <v/>
-      </c>
-      <c r="E31" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D31))</f>
-        <v/>
-      </c>
-      <c r="F31" s="10">
-        <f>E31-E30</f>
-        <v/>
-      </c>
-      <c r="G31" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E31),0)</f>
+        <f>C31*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E31" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B31),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F31" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B31,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G31" s="12">
+        <f>C31-F31</f>
         <v/>
       </c>
       <c r="H31" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E31,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I31" s="12">
-        <f>G31-H31</f>
-        <v/>
-      </c>
-      <c r="J31" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E31),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K31" s="12">
-        <f>D31-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E31),0)</f>
+        <f>H30+E31</f>
+        <v/>
+      </c>
+      <c r="I31" s="10">
+        <f>B31-B30</f>
+        <v/>
+      </c>
+      <c r="J31" s="12">
+        <f>E31</f>
         <v/>
       </c>
     </row>
@@ -13074,44 +12948,40 @@
       <c r="A32" s="10" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="12">
-        <f>G31</f>
-        <v/>
-      </c>
-      <c r="C32" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E31),0))*Paramètres!$B$3</f>
+      <c r="B32" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H31))</f>
+        <v/>
+      </c>
+      <c r="C32" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B32),0)</f>
         <v/>
       </c>
       <c r="D32" s="12">
-        <f>D31+C32</f>
-        <v/>
-      </c>
-      <c r="E32" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D32))</f>
-        <v/>
-      </c>
-      <c r="F32" s="10">
-        <f>E32-E31</f>
-        <v/>
-      </c>
-      <c r="G32" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E32),0)</f>
+        <f>C32*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E32" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B32),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F32" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B32,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G32" s="12">
+        <f>C32-F32</f>
         <v/>
       </c>
       <c r="H32" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E32,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I32" s="12">
-        <f>G32-H32</f>
-        <v/>
-      </c>
-      <c r="J32" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E32),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K32" s="12">
-        <f>D32-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E32),0)</f>
+        <f>H31+E32</f>
+        <v/>
+      </c>
+      <c r="I32" s="10">
+        <f>B32-B31</f>
+        <v/>
+      </c>
+      <c r="J32" s="12">
+        <f>E32</f>
         <v/>
       </c>
     </row>
@@ -13119,44 +12989,40 @@
       <c r="A33" s="10" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="12">
-        <f>G32</f>
-        <v/>
-      </c>
-      <c r="C33" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E32),0))*Paramètres!$B$3</f>
+      <c r="B33" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H32))</f>
+        <v/>
+      </c>
+      <c r="C33" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B33),0)</f>
         <v/>
       </c>
       <c r="D33" s="12">
-        <f>D32+C33</f>
-        <v/>
-      </c>
-      <c r="E33" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D33))</f>
-        <v/>
-      </c>
-      <c r="F33" s="10">
-        <f>E33-E32</f>
-        <v/>
-      </c>
-      <c r="G33" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E33),0)</f>
+        <f>C33*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E33" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B33),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F33" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B33,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G33" s="12">
+        <f>C33-F33</f>
         <v/>
       </c>
       <c r="H33" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E33,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I33" s="12">
-        <f>G33-H33</f>
-        <v/>
-      </c>
-      <c r="J33" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E33),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K33" s="12">
-        <f>D33-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E33),0)</f>
+        <f>H32+E33</f>
+        <v/>
+      </c>
+      <c r="I33" s="10">
+        <f>B33-B32</f>
+        <v/>
+      </c>
+      <c r="J33" s="12">
+        <f>E33</f>
         <v/>
       </c>
     </row>
@@ -13164,44 +13030,40 @@
       <c r="A34" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="12">
-        <f>G33</f>
-        <v/>
-      </c>
-      <c r="C34" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E33),0))*Paramètres!$B$3</f>
+      <c r="B34" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H33))</f>
+        <v/>
+      </c>
+      <c r="C34" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B34),0)</f>
         <v/>
       </c>
       <c r="D34" s="12">
-        <f>D33+C34</f>
-        <v/>
-      </c>
-      <c r="E34" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D34))</f>
-        <v/>
-      </c>
-      <c r="F34" s="10">
-        <f>E34-E33</f>
-        <v/>
-      </c>
-      <c r="G34" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E34),0)</f>
+        <f>C34*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E34" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B34),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F34" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B34,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G34" s="12">
+        <f>C34-F34</f>
         <v/>
       </c>
       <c r="H34" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E34,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I34" s="12">
-        <f>G34-H34</f>
-        <v/>
-      </c>
-      <c r="J34" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E34),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K34" s="12">
-        <f>D34-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E34),0)</f>
+        <f>H33+E34</f>
+        <v/>
+      </c>
+      <c r="I34" s="10">
+        <f>B34-B33</f>
+        <v/>
+      </c>
+      <c r="J34" s="12">
+        <f>E34</f>
         <v/>
       </c>
     </row>
@@ -13209,44 +13071,40 @@
       <c r="A35" s="10" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="12">
-        <f>G34</f>
-        <v/>
-      </c>
-      <c r="C35" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E34),0))*Paramètres!$B$3</f>
+      <c r="B35" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H34))</f>
+        <v/>
+      </c>
+      <c r="C35" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B35),0)</f>
         <v/>
       </c>
       <c r="D35" s="12">
-        <f>D34+C35</f>
-        <v/>
-      </c>
-      <c r="E35" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D35))</f>
-        <v/>
-      </c>
-      <c r="F35" s="10">
-        <f>E35-E34</f>
-        <v/>
-      </c>
-      <c r="G35" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E35),0)</f>
+        <f>C35*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E35" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B35),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F35" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B35,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G35" s="12">
+        <f>C35-F35</f>
         <v/>
       </c>
       <c r="H35" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E35,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I35" s="12">
-        <f>G35-H35</f>
-        <v/>
-      </c>
-      <c r="J35" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E35),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K35" s="12">
-        <f>D35-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E35),0)</f>
+        <f>H34+E35</f>
+        <v/>
+      </c>
+      <c r="I35" s="10">
+        <f>B35-B34</f>
+        <v/>
+      </c>
+      <c r="J35" s="12">
+        <f>E35</f>
         <v/>
       </c>
     </row>
@@ -13254,44 +13112,40 @@
       <c r="A36" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="12">
-        <f>G35</f>
-        <v/>
-      </c>
-      <c r="C36" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E35),0))*Paramètres!$B$3</f>
+      <c r="B36" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H35))</f>
+        <v/>
+      </c>
+      <c r="C36" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B36),0)</f>
         <v/>
       </c>
       <c r="D36" s="12">
-        <f>D35+C36</f>
-        <v/>
-      </c>
-      <c r="E36" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D36))</f>
-        <v/>
-      </c>
-      <c r="F36" s="10">
-        <f>E36-E35</f>
-        <v/>
-      </c>
-      <c r="G36" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E36),0)</f>
+        <f>C36*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E36" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B36),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F36" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B36,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G36" s="12">
+        <f>C36-F36</f>
         <v/>
       </c>
       <c r="H36" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E36,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I36" s="12">
-        <f>G36-H36</f>
-        <v/>
-      </c>
-      <c r="J36" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E36),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K36" s="12">
-        <f>D36-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E36),0)</f>
+        <f>H35+E36</f>
+        <v/>
+      </c>
+      <c r="I36" s="10">
+        <f>B36-B35</f>
+        <v/>
+      </c>
+      <c r="J36" s="12">
+        <f>E36</f>
         <v/>
       </c>
     </row>
@@ -13299,44 +13153,40 @@
       <c r="A37" s="10" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="12">
-        <f>G36</f>
-        <v/>
-      </c>
-      <c r="C37" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E36),0))*Paramètres!$B$3</f>
+      <c r="B37" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H36))</f>
+        <v/>
+      </c>
+      <c r="C37" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B37),0)</f>
         <v/>
       </c>
       <c r="D37" s="12">
-        <f>D36+C37</f>
-        <v/>
-      </c>
-      <c r="E37" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D37))</f>
-        <v/>
-      </c>
-      <c r="F37" s="10">
-        <f>E37-E36</f>
-        <v/>
-      </c>
-      <c r="G37" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E37),0)</f>
+        <f>C37*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E37" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B37),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F37" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B37,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G37" s="12">
+        <f>C37-F37</f>
         <v/>
       </c>
       <c r="H37" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E37,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I37" s="12">
-        <f>G37-H37</f>
-        <v/>
-      </c>
-      <c r="J37" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E37),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K37" s="12">
-        <f>D37-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E37),0)</f>
+        <f>H36+E37</f>
+        <v/>
+      </c>
+      <c r="I37" s="10">
+        <f>B37-B36</f>
+        <v/>
+      </c>
+      <c r="J37" s="12">
+        <f>E37</f>
         <v/>
       </c>
     </row>
@@ -13344,44 +13194,40 @@
       <c r="A38" s="10" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="12">
-        <f>G37</f>
-        <v/>
-      </c>
-      <c r="C38" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E37),0))*Paramètres!$B$3</f>
+      <c r="B38" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H37))</f>
+        <v/>
+      </c>
+      <c r="C38" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B38),0)</f>
         <v/>
       </c>
       <c r="D38" s="12">
-        <f>D37+C38</f>
-        <v/>
-      </c>
-      <c r="E38" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D38))</f>
-        <v/>
-      </c>
-      <c r="F38" s="10">
-        <f>E38-E37</f>
-        <v/>
-      </c>
-      <c r="G38" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E38),0)</f>
+        <f>C38*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E38" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B38),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F38" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B38,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G38" s="12">
+        <f>C38-F38</f>
         <v/>
       </c>
       <c r="H38" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E38,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I38" s="12">
-        <f>G38-H38</f>
-        <v/>
-      </c>
-      <c r="J38" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E38),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K38" s="12">
-        <f>D38-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E38),0)</f>
+        <f>H37+E38</f>
+        <v/>
+      </c>
+      <c r="I38" s="10">
+        <f>B38-B37</f>
+        <v/>
+      </c>
+      <c r="J38" s="12">
+        <f>E38</f>
         <v/>
       </c>
     </row>
@@ -13389,44 +13235,40 @@
       <c r="A39" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="12">
-        <f>G38</f>
-        <v/>
-      </c>
-      <c r="C39" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E38),0))*Paramètres!$B$3</f>
+      <c r="B39" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H38))</f>
+        <v/>
+      </c>
+      <c r="C39" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B39),0)</f>
         <v/>
       </c>
       <c r="D39" s="12">
-        <f>D38+C39</f>
-        <v/>
-      </c>
-      <c r="E39" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D39))</f>
-        <v/>
-      </c>
-      <c r="F39" s="10">
-        <f>E39-E38</f>
-        <v/>
-      </c>
-      <c r="G39" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E39),0)</f>
+        <f>C39*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E39" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B39),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F39" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B39,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G39" s="12">
+        <f>C39-F39</f>
         <v/>
       </c>
       <c r="H39" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E39,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I39" s="12">
-        <f>G39-H39</f>
-        <v/>
-      </c>
-      <c r="J39" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E39),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K39" s="12">
-        <f>D39-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E39),0)</f>
+        <f>H38+E39</f>
+        <v/>
+      </c>
+      <c r="I39" s="10">
+        <f>B39-B38</f>
+        <v/>
+      </c>
+      <c r="J39" s="12">
+        <f>E39</f>
         <v/>
       </c>
     </row>
@@ -13434,44 +13276,40 @@
       <c r="A40" s="10" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="12">
-        <f>G39</f>
-        <v/>
-      </c>
-      <c r="C40" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E39),0))*Paramètres!$B$3</f>
+      <c r="B40" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H39))</f>
+        <v/>
+      </c>
+      <c r="C40" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B40),0)</f>
         <v/>
       </c>
       <c r="D40" s="12">
-        <f>D39+C40</f>
-        <v/>
-      </c>
-      <c r="E40" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D40))</f>
-        <v/>
-      </c>
-      <c r="F40" s="10">
-        <f>E40-E39</f>
-        <v/>
-      </c>
-      <c r="G40" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E40),0)</f>
+        <f>C40*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E40" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B40),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F40" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B40,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G40" s="12">
+        <f>C40-F40</f>
         <v/>
       </c>
       <c r="H40" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E40,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I40" s="12">
-        <f>G40-H40</f>
-        <v/>
-      </c>
-      <c r="J40" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E40),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K40" s="12">
-        <f>D40-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E40),0)</f>
+        <f>H39+E40</f>
+        <v/>
+      </c>
+      <c r="I40" s="10">
+        <f>B40-B39</f>
+        <v/>
+      </c>
+      <c r="J40" s="12">
+        <f>E40</f>
         <v/>
       </c>
     </row>
@@ -13479,44 +13317,40 @@
       <c r="A41" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="12">
-        <f>G40</f>
-        <v/>
-      </c>
-      <c r="C41" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E40),0))*Paramètres!$B$3</f>
+      <c r="B41" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H40))</f>
+        <v/>
+      </c>
+      <c r="C41" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B41),0)</f>
         <v/>
       </c>
       <c r="D41" s="12">
-        <f>D40+C41</f>
-        <v/>
-      </c>
-      <c r="E41" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D41))</f>
-        <v/>
-      </c>
-      <c r="F41" s="10">
-        <f>E41-E40</f>
-        <v/>
-      </c>
-      <c r="G41" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E41),0)</f>
+        <f>C41*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E41" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B41),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F41" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B41,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G41" s="12">
+        <f>C41-F41</f>
         <v/>
       </c>
       <c r="H41" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E41,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I41" s="12">
-        <f>G41-H41</f>
-        <v/>
-      </c>
-      <c r="J41" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E41),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K41" s="12">
-        <f>D41-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E41),0)</f>
+        <f>H40+E41</f>
+        <v/>
+      </c>
+      <c r="I41" s="10">
+        <f>B41-B40</f>
+        <v/>
+      </c>
+      <c r="J41" s="12">
+        <f>E41</f>
         <v/>
       </c>
     </row>
@@ -13524,44 +13358,40 @@
       <c r="A42" s="10" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="12">
-        <f>G41</f>
-        <v/>
-      </c>
-      <c r="C42" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E41),0))*Paramètres!$B$3</f>
+      <c r="B42" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H41))</f>
+        <v/>
+      </c>
+      <c r="C42" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B42),0)</f>
         <v/>
       </c>
       <c r="D42" s="12">
-        <f>D41+C42</f>
-        <v/>
-      </c>
-      <c r="E42" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D42))</f>
-        <v/>
-      </c>
-      <c r="F42" s="10">
-        <f>E42-E41</f>
-        <v/>
-      </c>
-      <c r="G42" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E42),0)</f>
+        <f>C42*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E42" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B42),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F42" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B42,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G42" s="12">
+        <f>C42-F42</f>
         <v/>
       </c>
       <c r="H42" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E42,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I42" s="12">
-        <f>G42-H42</f>
-        <v/>
-      </c>
-      <c r="J42" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E42),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K42" s="12">
-        <f>D42-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E42),0)</f>
+        <f>H41+E42</f>
+        <v/>
+      </c>
+      <c r="I42" s="10">
+        <f>B42-B41</f>
+        <v/>
+      </c>
+      <c r="J42" s="12">
+        <f>E42</f>
         <v/>
       </c>
     </row>
@@ -13569,44 +13399,40 @@
       <c r="A43" s="10" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="12">
-        <f>G42</f>
-        <v/>
-      </c>
-      <c r="C43" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E42),0))*Paramètres!$B$3</f>
+      <c r="B43" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H42))</f>
+        <v/>
+      </c>
+      <c r="C43" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B43),0)</f>
         <v/>
       </c>
       <c r="D43" s="12">
-        <f>D42+C43</f>
-        <v/>
-      </c>
-      <c r="E43" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D43))</f>
-        <v/>
-      </c>
-      <c r="F43" s="10">
-        <f>E43-E42</f>
-        <v/>
-      </c>
-      <c r="G43" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E43),0)</f>
+        <f>C43*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E43" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B43),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F43" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B43,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G43" s="12">
+        <f>C43-F43</f>
         <v/>
       </c>
       <c r="H43" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E43,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I43" s="12">
-        <f>G43-H43</f>
-        <v/>
-      </c>
-      <c r="J43" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E43),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K43" s="12">
-        <f>D43-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E43),0)</f>
+        <f>H42+E43</f>
+        <v/>
+      </c>
+      <c r="I43" s="10">
+        <f>B43-B42</f>
+        <v/>
+      </c>
+      <c r="J43" s="12">
+        <f>E43</f>
         <v/>
       </c>
     </row>
@@ -13614,44 +13440,40 @@
       <c r="A44" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="12">
-        <f>G43</f>
-        <v/>
-      </c>
-      <c r="C44" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E43),0))*Paramètres!$B$3</f>
+      <c r="B44" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H43))</f>
+        <v/>
+      </c>
+      <c r="C44" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B44),0)</f>
         <v/>
       </c>
       <c r="D44" s="12">
-        <f>D43+C44</f>
-        <v/>
-      </c>
-      <c r="E44" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D44))</f>
-        <v/>
-      </c>
-      <c r="F44" s="10">
-        <f>E44-E43</f>
-        <v/>
-      </c>
-      <c r="G44" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E44),0)</f>
+        <f>C44*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E44" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B44),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F44" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B44,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G44" s="12">
+        <f>C44-F44</f>
         <v/>
       </c>
       <c r="H44" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E44,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I44" s="12">
-        <f>G44-H44</f>
-        <v/>
-      </c>
-      <c r="J44" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E44),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K44" s="12">
-        <f>D44-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E44),0)</f>
+        <f>H43+E44</f>
+        <v/>
+      </c>
+      <c r="I44" s="10">
+        <f>B44-B43</f>
+        <v/>
+      </c>
+      <c r="J44" s="12">
+        <f>E44</f>
         <v/>
       </c>
     </row>
@@ -13659,44 +13481,40 @@
       <c r="A45" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="12">
-        <f>G44</f>
-        <v/>
-      </c>
-      <c r="C45" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E44),0))*Paramètres!$B$3</f>
+      <c r="B45" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H44))</f>
+        <v/>
+      </c>
+      <c r="C45" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B45),0)</f>
         <v/>
       </c>
       <c r="D45" s="12">
-        <f>D44+C45</f>
-        <v/>
-      </c>
-      <c r="E45" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D45))</f>
-        <v/>
-      </c>
-      <c r="F45" s="10">
-        <f>E45-E44</f>
-        <v/>
-      </c>
-      <c r="G45" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E45),0)</f>
+        <f>C45*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E45" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B45),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F45" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B45,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G45" s="12">
+        <f>C45-F45</f>
         <v/>
       </c>
       <c r="H45" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E45,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I45" s="12">
-        <f>G45-H45</f>
-        <v/>
-      </c>
-      <c r="J45" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E45),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K45" s="12">
-        <f>D45-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E45),0)</f>
+        <f>H44+E45</f>
+        <v/>
+      </c>
+      <c r="I45" s="10">
+        <f>B45-B44</f>
+        <v/>
+      </c>
+      <c r="J45" s="12">
+        <f>E45</f>
         <v/>
       </c>
     </row>
@@ -13704,44 +13522,40 @@
       <c r="A46" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="12">
-        <f>G45</f>
-        <v/>
-      </c>
-      <c r="C46" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E45),0))*Paramètres!$B$3</f>
+      <c r="B46" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H45))</f>
+        <v/>
+      </c>
+      <c r="C46" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B46),0)</f>
         <v/>
       </c>
       <c r="D46" s="12">
-        <f>D45+C46</f>
-        <v/>
-      </c>
-      <c r="E46" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D46))</f>
-        <v/>
-      </c>
-      <c r="F46" s="10">
-        <f>E46-E45</f>
-        <v/>
-      </c>
-      <c r="G46" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E46),0)</f>
+        <f>C46*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E46" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B46),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F46" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B46,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G46" s="12">
+        <f>C46-F46</f>
         <v/>
       </c>
       <c r="H46" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E46,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I46" s="12">
-        <f>G46-H46</f>
-        <v/>
-      </c>
-      <c r="J46" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E46),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K46" s="12">
-        <f>D46-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E46),0)</f>
+        <f>H45+E46</f>
+        <v/>
+      </c>
+      <c r="I46" s="10">
+        <f>B46-B45</f>
+        <v/>
+      </c>
+      <c r="J46" s="12">
+        <f>E46</f>
         <v/>
       </c>
     </row>
@@ -13749,44 +13563,40 @@
       <c r="A47" s="10" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="12">
-        <f>G46</f>
-        <v/>
-      </c>
-      <c r="C47" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E46),0))*Paramètres!$B$3</f>
+      <c r="B47" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H46))</f>
+        <v/>
+      </c>
+      <c r="C47" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B47),0)</f>
         <v/>
       </c>
       <c r="D47" s="12">
-        <f>D46+C47</f>
-        <v/>
-      </c>
-      <c r="E47" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D47))</f>
-        <v/>
-      </c>
-      <c r="F47" s="10">
-        <f>E47-E46</f>
-        <v/>
-      </c>
-      <c r="G47" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E47),0)</f>
+        <f>C47*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E47" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B47),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F47" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B47,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G47" s="12">
+        <f>C47-F47</f>
         <v/>
       </c>
       <c r="H47" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E47,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I47" s="12">
-        <f>G47-H47</f>
-        <v/>
-      </c>
-      <c r="J47" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E47),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K47" s="12">
-        <f>D47-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E47),0)</f>
+        <f>H46+E47</f>
+        <v/>
+      </c>
+      <c r="I47" s="10">
+        <f>B47-B46</f>
+        <v/>
+      </c>
+      <c r="J47" s="12">
+        <f>E47</f>
         <v/>
       </c>
     </row>
@@ -13794,44 +13604,40 @@
       <c r="A48" s="10" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="12">
-        <f>G47</f>
-        <v/>
-      </c>
-      <c r="C48" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E47),0))*Paramètres!$B$3</f>
+      <c r="B48" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H47))</f>
+        <v/>
+      </c>
+      <c r="C48" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B48),0)</f>
         <v/>
       </c>
       <c r="D48" s="12">
-        <f>D47+C48</f>
-        <v/>
-      </c>
-      <c r="E48" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D48))</f>
-        <v/>
-      </c>
-      <c r="F48" s="10">
-        <f>E48-E47</f>
-        <v/>
-      </c>
-      <c r="G48" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E48),0)</f>
+        <f>C48*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E48" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B48),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F48" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B48,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G48" s="12">
+        <f>C48-F48</f>
         <v/>
       </c>
       <c r="H48" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E48,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I48" s="12">
-        <f>G48-H48</f>
-        <v/>
-      </c>
-      <c r="J48" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E48),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K48" s="12">
-        <f>D48-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E48),0)</f>
+        <f>H47+E48</f>
+        <v/>
+      </c>
+      <c r="I48" s="10">
+        <f>B48-B47</f>
+        <v/>
+      </c>
+      <c r="J48" s="12">
+        <f>E48</f>
         <v/>
       </c>
     </row>
@@ -13839,44 +13645,40 @@
       <c r="A49" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="12">
-        <f>G48</f>
-        <v/>
-      </c>
-      <c r="C49" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E48),0))*Paramètres!$B$3</f>
+      <c r="B49" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H48))</f>
+        <v/>
+      </c>
+      <c r="C49" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B49),0)</f>
         <v/>
       </c>
       <c r="D49" s="12">
-        <f>D48+C49</f>
-        <v/>
-      </c>
-      <c r="E49" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D49))</f>
-        <v/>
-      </c>
-      <c r="F49" s="10">
-        <f>E49-E48</f>
-        <v/>
-      </c>
-      <c r="G49" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E49),0)</f>
+        <f>C49*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E49" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B49),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F49" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B49,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G49" s="12">
+        <f>C49-F49</f>
         <v/>
       </c>
       <c r="H49" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E49,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I49" s="12">
-        <f>G49-H49</f>
-        <v/>
-      </c>
-      <c r="J49" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E49),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K49" s="12">
-        <f>D49-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E49),0)</f>
+        <f>H48+E49</f>
+        <v/>
+      </c>
+      <c r="I49" s="10">
+        <f>B49-B48</f>
+        <v/>
+      </c>
+      <c r="J49" s="12">
+        <f>E49</f>
         <v/>
       </c>
     </row>
@@ -13884,44 +13686,40 @@
       <c r="A50" s="10" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="12">
-        <f>G49</f>
-        <v/>
-      </c>
-      <c r="C50" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E49),0))*Paramètres!$B$3</f>
+      <c r="B50" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H49))</f>
+        <v/>
+      </c>
+      <c r="C50" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B50),0)</f>
         <v/>
       </c>
       <c r="D50" s="12">
-        <f>D49+C50</f>
-        <v/>
-      </c>
-      <c r="E50" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D50))</f>
-        <v/>
-      </c>
-      <c r="F50" s="10">
-        <f>E50-E49</f>
-        <v/>
-      </c>
-      <c r="G50" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E50),0)</f>
+        <f>C50*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E50" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B50),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F50" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B50,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G50" s="12">
+        <f>C50-F50</f>
         <v/>
       </c>
       <c r="H50" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E50,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I50" s="12">
-        <f>G50-H50</f>
-        <v/>
-      </c>
-      <c r="J50" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E50),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K50" s="12">
-        <f>D50-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E50),0)</f>
+        <f>H49+E50</f>
+        <v/>
+      </c>
+      <c r="I50" s="10">
+        <f>B50-B49</f>
+        <v/>
+      </c>
+      <c r="J50" s="12">
+        <f>E50</f>
         <v/>
       </c>
     </row>
@@ -13929,44 +13727,40 @@
       <c r="A51" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="12">
-        <f>G50</f>
-        <v/>
-      </c>
-      <c r="C51" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E50),0))*Paramètres!$B$3</f>
+      <c r="B51" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H50))</f>
+        <v/>
+      </c>
+      <c r="C51" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B51),0)</f>
         <v/>
       </c>
       <c r="D51" s="12">
-        <f>D50+C51</f>
-        <v/>
-      </c>
-      <c r="E51" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D51))</f>
-        <v/>
-      </c>
-      <c r="F51" s="10">
-        <f>E51-E50</f>
-        <v/>
-      </c>
-      <c r="G51" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E51),0)</f>
+        <f>C51*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E51" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B51),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F51" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B51,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G51" s="12">
+        <f>C51-F51</f>
         <v/>
       </c>
       <c r="H51" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E51,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I51" s="12">
-        <f>G51-H51</f>
-        <v/>
-      </c>
-      <c r="J51" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E51),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K51" s="12">
-        <f>D51-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E51),0)</f>
+        <f>H50+E51</f>
+        <v/>
+      </c>
+      <c r="I51" s="10">
+        <f>B51-B50</f>
+        <v/>
+      </c>
+      <c r="J51" s="12">
+        <f>E51</f>
         <v/>
       </c>
     </row>
@@ -13974,44 +13768,40 @@
       <c r="A52" s="10" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="12">
-        <f>G51</f>
-        <v/>
-      </c>
-      <c r="C52" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E51),0))*Paramètres!$B$3</f>
+      <c r="B52" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H51))</f>
+        <v/>
+      </c>
+      <c r="C52" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B52),0)</f>
         <v/>
       </c>
       <c r="D52" s="12">
-        <f>D51+C52</f>
-        <v/>
-      </c>
-      <c r="E52" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D52))</f>
-        <v/>
-      </c>
-      <c r="F52" s="10">
-        <f>E52-E51</f>
-        <v/>
-      </c>
-      <c r="G52" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E52),0)</f>
+        <f>C52*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E52" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B52),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F52" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B52,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G52" s="12">
+        <f>C52-F52</f>
         <v/>
       </c>
       <c r="H52" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E52,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I52" s="12">
-        <f>G52-H52</f>
-        <v/>
-      </c>
-      <c r="J52" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E52),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K52" s="12">
-        <f>D52-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E52),0)</f>
+        <f>H51+E52</f>
+        <v/>
+      </c>
+      <c r="I52" s="10">
+        <f>B52-B51</f>
+        <v/>
+      </c>
+      <c r="J52" s="12">
+        <f>E52</f>
         <v/>
       </c>
     </row>
@@ -14019,44 +13809,40 @@
       <c r="A53" s="10" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="12">
-        <f>G52</f>
-        <v/>
-      </c>
-      <c r="C53" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E52),0))*Paramètres!$B$3</f>
+      <c r="B53" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H52))</f>
+        <v/>
+      </c>
+      <c r="C53" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B53),0)</f>
         <v/>
       </c>
       <c r="D53" s="12">
-        <f>D52+C53</f>
-        <v/>
-      </c>
-      <c r="E53" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D53))</f>
-        <v/>
-      </c>
-      <c r="F53" s="10">
-        <f>E53-E52</f>
-        <v/>
-      </c>
-      <c r="G53" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E53),0)</f>
+        <f>C53*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E53" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B53),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F53" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B53,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G53" s="12">
+        <f>C53-F53</f>
         <v/>
       </c>
       <c r="H53" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E53,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I53" s="12">
-        <f>G53-H53</f>
-        <v/>
-      </c>
-      <c r="J53" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E53),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K53" s="12">
-        <f>D53-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E53),0)</f>
+        <f>H52+E53</f>
+        <v/>
+      </c>
+      <c r="I53" s="10">
+        <f>B53-B52</f>
+        <v/>
+      </c>
+      <c r="J53" s="12">
+        <f>E53</f>
         <v/>
       </c>
     </row>
@@ -14064,44 +13850,40 @@
       <c r="A54" s="10" t="n">
         <v>53</v>
       </c>
-      <c r="B54" s="12">
-        <f>G53</f>
-        <v/>
-      </c>
-      <c r="C54" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E53),0))*Paramètres!$B$3</f>
+      <c r="B54" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H53))</f>
+        <v/>
+      </c>
+      <c r="C54" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B54),0)</f>
         <v/>
       </c>
       <c r="D54" s="12">
-        <f>D53+C54</f>
-        <v/>
-      </c>
-      <c r="E54" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D54))</f>
-        <v/>
-      </c>
-      <c r="F54" s="10">
-        <f>E54-E53</f>
-        <v/>
-      </c>
-      <c r="G54" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E54),0)</f>
+        <f>C54*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E54" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B54),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F54" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B54,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G54" s="12">
+        <f>C54-F54</f>
         <v/>
       </c>
       <c r="H54" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E54,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I54" s="12">
-        <f>G54-H54</f>
-        <v/>
-      </c>
-      <c r="J54" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E54),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K54" s="12">
-        <f>D54-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E54),0)</f>
+        <f>H53+E54</f>
+        <v/>
+      </c>
+      <c r="I54" s="10">
+        <f>B54-B53</f>
+        <v/>
+      </c>
+      <c r="J54" s="12">
+        <f>E54</f>
         <v/>
       </c>
     </row>
@@ -14109,44 +13891,40 @@
       <c r="A55" s="10" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="12">
-        <f>G54</f>
-        <v/>
-      </c>
-      <c r="C55" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E54),0))*Paramètres!$B$3</f>
+      <c r="B55" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H54))</f>
+        <v/>
+      </c>
+      <c r="C55" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B55),0)</f>
         <v/>
       </c>
       <c r="D55" s="12">
-        <f>D54+C55</f>
-        <v/>
-      </c>
-      <c r="E55" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D55))</f>
-        <v/>
-      </c>
-      <c r="F55" s="10">
-        <f>E55-E54</f>
-        <v/>
-      </c>
-      <c r="G55" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E55),0)</f>
+        <f>C55*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E55" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B55),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F55" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B55,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G55" s="12">
+        <f>C55-F55</f>
         <v/>
       </c>
       <c r="H55" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E55,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I55" s="12">
-        <f>G55-H55</f>
-        <v/>
-      </c>
-      <c r="J55" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E55),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K55" s="12">
-        <f>D55-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E55),0)</f>
+        <f>H54+E55</f>
+        <v/>
+      </c>
+      <c r="I55" s="10">
+        <f>B55-B54</f>
+        <v/>
+      </c>
+      <c r="J55" s="12">
+        <f>E55</f>
         <v/>
       </c>
     </row>
@@ -14154,44 +13932,40 @@
       <c r="A56" s="10" t="n">
         <v>55</v>
       </c>
-      <c r="B56" s="12">
-        <f>G55</f>
-        <v/>
-      </c>
-      <c r="C56" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E55),0))*Paramètres!$B$3</f>
+      <c r="B56" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H55))</f>
+        <v/>
+      </c>
+      <c r="C56" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B56),0)</f>
         <v/>
       </c>
       <c r="D56" s="12">
-        <f>D55+C56</f>
-        <v/>
-      </c>
-      <c r="E56" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D56))</f>
-        <v/>
-      </c>
-      <c r="F56" s="10">
-        <f>E56-E55</f>
-        <v/>
-      </c>
-      <c r="G56" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E56),0)</f>
+        <f>C56*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E56" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B56),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F56" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B56,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G56" s="12">
+        <f>C56-F56</f>
         <v/>
       </c>
       <c r="H56" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E56,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I56" s="12">
-        <f>G56-H56</f>
-        <v/>
-      </c>
-      <c r="J56" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E56),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K56" s="12">
-        <f>D56-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E56),0)</f>
+        <f>H55+E56</f>
+        <v/>
+      </c>
+      <c r="I56" s="10">
+        <f>B56-B55</f>
+        <v/>
+      </c>
+      <c r="J56" s="12">
+        <f>E56</f>
         <v/>
       </c>
     </row>
@@ -14199,44 +13973,40 @@
       <c r="A57" s="10" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="12">
-        <f>G56</f>
-        <v/>
-      </c>
-      <c r="C57" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E56),0))*Paramètres!$B$3</f>
+      <c r="B57" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H56))</f>
+        <v/>
+      </c>
+      <c r="C57" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B57),0)</f>
         <v/>
       </c>
       <c r="D57" s="12">
-        <f>D56+C57</f>
-        <v/>
-      </c>
-      <c r="E57" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D57))</f>
-        <v/>
-      </c>
-      <c r="F57" s="10">
-        <f>E57-E56</f>
-        <v/>
-      </c>
-      <c r="G57" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E57),0)</f>
+        <f>C57*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E57" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B57),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F57" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B57,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G57" s="12">
+        <f>C57-F57</f>
         <v/>
       </c>
       <c r="H57" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E57,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I57" s="12">
-        <f>G57-H57</f>
-        <v/>
-      </c>
-      <c r="J57" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E57),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K57" s="12">
-        <f>D57-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E57),0)</f>
+        <f>H56+E57</f>
+        <v/>
+      </c>
+      <c r="I57" s="10">
+        <f>B57-B56</f>
+        <v/>
+      </c>
+      <c r="J57" s="12">
+        <f>E57</f>
         <v/>
       </c>
     </row>
@@ -14244,44 +14014,40 @@
       <c r="A58" s="10" t="n">
         <v>57</v>
       </c>
-      <c r="B58" s="12">
-        <f>G57</f>
-        <v/>
-      </c>
-      <c r="C58" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E57),0))*Paramètres!$B$3</f>
+      <c r="B58" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H57))</f>
+        <v/>
+      </c>
+      <c r="C58" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B58),0)</f>
         <v/>
       </c>
       <c r="D58" s="12">
-        <f>D57+C58</f>
-        <v/>
-      </c>
-      <c r="E58" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D58))</f>
-        <v/>
-      </c>
-      <c r="F58" s="10">
-        <f>E58-E57</f>
-        <v/>
-      </c>
-      <c r="G58" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E58),0)</f>
+        <f>C58*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E58" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B58),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F58" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B58,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G58" s="12">
+        <f>C58-F58</f>
         <v/>
       </c>
       <c r="H58" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E58,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I58" s="12">
-        <f>G58-H58</f>
-        <v/>
-      </c>
-      <c r="J58" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E58),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K58" s="12">
-        <f>D58-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E58),0)</f>
+        <f>H57+E58</f>
+        <v/>
+      </c>
+      <c r="I58" s="10">
+        <f>B58-B57</f>
+        <v/>
+      </c>
+      <c r="J58" s="12">
+        <f>E58</f>
         <v/>
       </c>
     </row>
@@ -14289,44 +14055,40 @@
       <c r="A59" s="10" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="12">
-        <f>G58</f>
-        <v/>
-      </c>
-      <c r="C59" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E58),0))*Paramètres!$B$3</f>
+      <c r="B59" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H58))</f>
+        <v/>
+      </c>
+      <c r="C59" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B59),0)</f>
         <v/>
       </c>
       <c r="D59" s="12">
-        <f>D58+C59</f>
-        <v/>
-      </c>
-      <c r="E59" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D59))</f>
-        <v/>
-      </c>
-      <c r="F59" s="10">
-        <f>E59-E58</f>
-        <v/>
-      </c>
-      <c r="G59" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E59),0)</f>
+        <f>C59*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E59" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B59),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F59" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B59,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G59" s="12">
+        <f>C59-F59</f>
         <v/>
       </c>
       <c r="H59" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E59,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I59" s="12">
-        <f>G59-H59</f>
-        <v/>
-      </c>
-      <c r="J59" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E59),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K59" s="12">
-        <f>D59-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E59),0)</f>
+        <f>H58+E59</f>
+        <v/>
+      </c>
+      <c r="I59" s="10">
+        <f>B59-B58</f>
+        <v/>
+      </c>
+      <c r="J59" s="12">
+        <f>E59</f>
         <v/>
       </c>
     </row>
@@ -14334,44 +14096,40 @@
       <c r="A60" s="10" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="12">
-        <f>G59</f>
-        <v/>
-      </c>
-      <c r="C60" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E59),0))*Paramètres!$B$3</f>
+      <c r="B60" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H59))</f>
+        <v/>
+      </c>
+      <c r="C60" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B60),0)</f>
         <v/>
       </c>
       <c r="D60" s="12">
-        <f>D59+C60</f>
-        <v/>
-      </c>
-      <c r="E60" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D60))</f>
-        <v/>
-      </c>
-      <c r="F60" s="10">
-        <f>E60-E59</f>
-        <v/>
-      </c>
-      <c r="G60" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E60),0)</f>
+        <f>C60*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E60" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B60),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F60" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B60,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G60" s="12">
+        <f>C60-F60</f>
         <v/>
       </c>
       <c r="H60" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E60,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I60" s="12">
-        <f>G60-H60</f>
-        <v/>
-      </c>
-      <c r="J60" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E60),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K60" s="12">
-        <f>D60-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E60),0)</f>
+        <f>H59+E60</f>
+        <v/>
+      </c>
+      <c r="I60" s="10">
+        <f>B60-B59</f>
+        <v/>
+      </c>
+      <c r="J60" s="12">
+        <f>E60</f>
         <v/>
       </c>
     </row>
@@ -14379,44 +14137,40 @@
       <c r="A61" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="12">
-        <f>G60</f>
-        <v/>
-      </c>
-      <c r="C61" s="12">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E60),0))*Paramètres!$B$3</f>
+      <c r="B61" s="10">
+        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;H60))</f>
+        <v/>
+      </c>
+      <c r="C61" s="16">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,B61),0)</f>
         <v/>
       </c>
       <c r="D61" s="12">
-        <f>D60+C61</f>
-        <v/>
-      </c>
-      <c r="E61" s="10">
-        <f>MIN(189,COUNTIF('Plan d''achat'!$K$2:$K$190,"&lt;="&amp;D61))</f>
-        <v/>
-      </c>
-      <c r="F61" s="10">
-        <f>E61-E60</f>
-        <v/>
-      </c>
-      <c r="G61" s="16">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,E61),0)</f>
+        <f>C61*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="E61" s="16">
+        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,B61),0))*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="F61" s="12">
+        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(B61,160)),0)</f>
+        <v/>
+      </c>
+      <c r="G61" s="12">
+        <f>C61-F61</f>
         <v/>
       </c>
       <c r="H61" s="12">
-        <f>Paramètres!$B$5+IFERROR(INDEX('Plan d''achat'!$I$2:$I$190,MIN(E61,160)),0)</f>
-        <v/>
-      </c>
-      <c r="I61" s="12">
-        <f>G61-H61</f>
-        <v/>
-      </c>
-      <c r="J61" s="16">
-        <f>(Paramètres!$B$5*(1-Paramètres!$B$4)+IFERROR(INDEX('Plan d''achat'!$J$2:$J$190,E61),0))*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="K61" s="12">
-        <f>D61-IFERROR(INDEX('Plan d''achat'!$K$2:$K$190,E61),0)</f>
+        <f>H60+E61</f>
+        <v/>
+      </c>
+      <c r="I61" s="10">
+        <f>B61-B60</f>
+        <v/>
+      </c>
+      <c r="J61" s="12">
+        <f>E61</f>
         <v/>
       </c>
     </row>

</xml_diff>